<commit_message>
feat: Updated GUI for dynamic route implementation
-Functionality to choose the destination route of the grades.
-Updated school logo on newsletter template and GUI.
-Improved GUI design: colors and icons implementation.
-Checking the EXCEL.EXE process to see if it is open or closed.
</commit_message>
<xml_diff>
--- a/Resource/BOLETIN.xlsx
+++ b/Resource/BOLETIN.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\Telegram Desktop\Proyecto-carlobranch\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\Proyecto\Resource\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACCD3513-6953-4680-B63B-4627F75ED8FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32A99FFC-1304-4550-9A2F-A9E5D6758244}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -382,38 +382,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -428,30 +405,79 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFFF99"/>
+      <color rgb="FFFFFFCC"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -468,22 +494,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>297366</xdr:colOff>
+      <xdr:colOff>254781</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>42559</xdr:rowOff>
+      <xdr:rowOff>28373</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>376363</xdr:colOff>
+      <xdr:colOff>346158</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>157976</xdr:rowOff>
+      <xdr:rowOff>170916</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
+        <xdr:cNvPr id="4" name="Imagen 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B0A8E7D7-3BC6-EE6D-8051-32E5836D58B6}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5BD0E5B5-0BEC-8020-B295-4F5BAB259CC8}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -505,8 +531,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="297366" y="42559"/>
-          <a:ext cx="785241" cy="659039"/>
+          <a:off x="254781" y="28373"/>
+          <a:ext cx="796632" cy="689724"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -849,404 +875,405 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="22"/>
+      <c r="A1" s="9"/>
       <c r="B1" s="10"/>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="10"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="31"/>
     </row>
     <row r="2" spans="1:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="13"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="34"/>
     </row>
     <row r="3" spans="1:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="16"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="36"/>
+      <c r="J3" s="36"/>
+      <c r="K3" s="37"/>
     </row>
     <row r="4" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="14"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="23" t="s">
+      <c r="A4" s="13"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="18"/>
-      <c r="K4" s="19"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="6"/>
     </row>
     <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="20" t="s">
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="18"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="7"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="3"/>
     </row>
     <row r="6" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="26" t="s">
+      <c r="A6" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="20" t="s">
+      <c r="B6" s="5"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="19"/>
-      <c r="F6" s="20" t="s">
+      <c r="E6" s="6"/>
+      <c r="F6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="20" t="s">
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="K6" s="19"/>
+      <c r="K6" s="6"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
+      <c r="A7" s="26"/>
+      <c r="B7" s="27"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
+      <c r="I7" s="27"/>
+      <c r="J7" s="27"/>
+      <c r="K7" s="28"/>
     </row>
     <row r="8" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="24" t="s">
+      <c r="A8" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="19"/>
-      <c r="H8" s="5" t="s">
+      <c r="B8" s="24"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="25"/>
+      <c r="H8" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="K8" s="5" t="s">
+      <c r="K8" s="39" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="21"/>
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="6"/>
+      <c r="A9" s="8"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="38"/>
+      <c r="I9" s="38"/>
+      <c r="J9" s="41"/>
+      <c r="K9" s="38"/>
     </row>
     <row r="10" spans="1:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17"/>
-      <c r="B10" s="18"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="6"/>
+      <c r="A10" s="4"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="38"/>
+      <c r="I10" s="38"/>
+      <c r="J10" s="41"/>
+      <c r="K10" s="38"/>
+      <c r="L10" s="42"/>
     </row>
     <row r="11" spans="1:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="17"/>
-      <c r="B11" s="18"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="6"/>
+      <c r="A11" s="4"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="38"/>
+      <c r="I11" s="38"/>
+      <c r="J11" s="41"/>
+      <c r="K11" s="38"/>
     </row>
     <row r="12" spans="1:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="17"/>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="19"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="6"/>
+      <c r="A12" s="4"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="38"/>
+      <c r="I12" s="38"/>
+      <c r="J12" s="41"/>
+      <c r="K12" s="38"/>
     </row>
     <row r="13" spans="1:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="17"/>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="19"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="6"/>
+      <c r="A13" s="4"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="38"/>
+      <c r="I13" s="38"/>
+      <c r="J13" s="41"/>
+      <c r="K13" s="38"/>
     </row>
     <row r="14" spans="1:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17"/>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="19"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="6"/>
+      <c r="A14" s="4"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="38"/>
+      <c r="I14" s="38"/>
+      <c r="J14" s="41"/>
+      <c r="K14" s="38"/>
     </row>
     <row r="15" spans="1:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="17"/>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="6"/>
+      <c r="A15" s="4"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="38"/>
+      <c r="I15" s="38"/>
+      <c r="J15" s="41"/>
+      <c r="K15" s="38"/>
     </row>
     <row r="16" spans="1:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17"/>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="6"/>
+      <c r="A16" s="4"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="38"/>
+      <c r="I16" s="38"/>
+      <c r="J16" s="41"/>
+      <c r="K16" s="38"/>
     </row>
     <row r="17" spans="1:11" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="17"/>
-      <c r="B17" s="18"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="6"/>
+      <c r="A17" s="4"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="38"/>
+      <c r="I17" s="38"/>
+      <c r="J17" s="41"/>
+      <c r="K17" s="38"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
     </row>
     <row r="20" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="27" t="s">
+      <c r="A20" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="3"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="20"/>
+      <c r="I20" s="20"/>
+      <c r="J20" s="20"/>
+      <c r="K20" s="1"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="4"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4"/>
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="4"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4"/>
-      <c r="J24" s="4"/>
-      <c r="K24" s="4"/>
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="4"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="4"/>
-      <c r="J25" s="4"/>
-      <c r="K25" s="4"/>
+      <c r="A25" s="2"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="4"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="28"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="28"/>
-      <c r="H26" s="15"/>
-      <c r="I26" s="15"/>
-      <c r="J26" s="4"/>
-      <c r="K26" s="4"/>
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="21"/>
+      <c r="H26" s="22"/>
+      <c r="I26" s="22"/>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
     </row>
     <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="4"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="25" t="s">
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="D27" s="9"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="25" t="s">
+      <c r="D27" s="17"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="H27" s="9"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="2"/>
+      <c r="K27" s="2"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A28" s="4"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
-      <c r="I28" s="4"/>
-      <c r="J28" s="4"/>
-      <c r="K28" s="4"/>
+      <c r="A28" s="2"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
+      <c r="K28" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="25">
     <mergeCell ref="C27:D27"/>
     <mergeCell ref="A16:G16"/>
     <mergeCell ref="A5:H5"/>
@@ -1271,6 +1298,7 @@
     <mergeCell ref="A1:B4"/>
     <mergeCell ref="C4:K4"/>
     <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A7:K7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.86" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" verticalDpi="300" r:id="rId1"/>

</xml_diff>